<commit_message>
Sincronizar datos acumulados (stock, salidas, costos, imágenes, caché)
Snapshots diarios de Stock/Salidas/Costos generados por corridas previas
del pipeline que no se habían guardado, más imágenes de producto y el
caché de Proyección Producción.
</commit_message>
<xml_diff>
--- a/Data/Productos/PRODUCTOS.xlsx
+++ b/Data/Productos/PRODUCTOS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SupplyDestileria\Documents\Bosque\Claude\Tablero operativo\Data\Productos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01016A06-2CB7-4DB9-B8FB-EA2469C603BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE60F89F-CA08-4A7A-B169-7497919C698E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{8FFC0A01-AC8B-4B89-A38C-E589AA3D5F39}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{8FFC0A01-AC8B-4B89-A38C-E589AA3D5F39}"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCTOS" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">INSUMOS!$A$2:$Q$79</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PRODUCTOS!$A$2:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PRODUCTOS!$A$2:$Q$130</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="320">
   <si>
     <t>RUBRO</t>
   </si>
@@ -905,12 +905,117 @@
   <si>
     <t>DECORMEC</t>
   </si>
+  <si>
+    <t>Bebidas</t>
+  </si>
+  <si>
+    <t>Estuche</t>
+  </si>
+  <si>
+    <t>Combo</t>
+  </si>
+  <si>
+    <t>Kit</t>
+  </si>
+  <si>
+    <t>Cristaleria</t>
+  </si>
+  <si>
+    <t>Indumentaria</t>
+  </si>
+  <si>
+    <t>Gorro Lana</t>
+  </si>
+  <si>
+    <t>Delantal</t>
+  </si>
+  <si>
+    <t>Mobiliario</t>
+  </si>
+  <si>
+    <t>Cartel</t>
+  </si>
+  <si>
+    <t>GINTONIC BOSQUE LATA X 269 ML X 6 UN</t>
+  </si>
+  <si>
+    <t>CAJON MORGADE 6 SIFONES SODA 1.5 LTS</t>
+  </si>
+  <si>
+    <t>FUNDA ARPILLERA BOSQUE</t>
+  </si>
+  <si>
+    <t>FUNDA LIENZO REFUGIOS</t>
+  </si>
+  <si>
+    <t>BOLSA DE ENTREGA BOSQUE 34X48X17</t>
+  </si>
+  <si>
+    <t>BOLSA DE ENTREGA BOSQUE 24X35X9</t>
+  </si>
+  <si>
+    <t>GIN BOSQUE NATIVO BOTELLA 500 ML + VASO BOSQUE TALLADO</t>
+  </si>
+  <si>
+    <t>GIN BOSQUE NATIVO BOTELLA 500 ML + VASO BOSQUE</t>
+  </si>
+  <si>
+    <t>KIT BOTANICOS X 6 - ESTUCHE MADERA</t>
+  </si>
+  <si>
+    <t>KIT BOTANICOS X 8 - ESTUCHE MADERA</t>
+  </si>
+  <si>
+    <t>MIX BOTÁNICOS X 6 - FUNDA LIENZO BOSQUE</t>
+  </si>
+  <si>
+    <t>KIT PRO COCTELERIA BY MONA GALLOSI</t>
+  </si>
+  <si>
+    <t>KIT FERIADO</t>
+  </si>
+  <si>
+    <t>DELANTAL BOSQUE</t>
+  </si>
+  <si>
+    <t>GORRO BOSQUE BY PHAROS - CLÁSICO BORDO</t>
+  </si>
+  <si>
+    <t>GORRO BOSQUE BY PHAROS - CLÁSICO GRIS</t>
+  </si>
+  <si>
+    <t>GORRO BOSQUE BY PHAROS - CLÁSICO NEGRO</t>
+  </si>
+  <si>
+    <t>CARTEL MADERA BOSQUE</t>
+  </si>
+  <si>
+    <t>SODA</t>
+  </si>
+  <si>
+    <t>GINTONIC</t>
+  </si>
+  <si>
+    <t>ARPILLERA</t>
+  </si>
+  <si>
+    <t>BOTANICOS</t>
+  </si>
+  <si>
+    <t>BOLSAS</t>
+  </si>
+  <si>
+    <t>PAPEL</t>
+  </si>
+  <si>
+    <t>LINEA CLASICA</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <color theme="1"/>
@@ -933,12 +1038,6 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -969,7 +1068,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1065,39 +1164,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1130,27 +1203,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1172,9 +1226,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1212,7 +1266,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1318,7 +1372,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1460,7 +1514,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1468,16 +1522,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9157580D-EE50-43E2-A76D-B56C98A189DD}">
-  <dimension ref="A1:Q92"/>
+  <dimension ref="A1:Q130"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="64.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="94.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12.75" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -1530,49 +1594,49 @@
       <c r="P2" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="Q2" s="18" t="s">
+      <c r="Q2" s="12" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="15">
-        <v>110036</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="17"/>
-      <c r="O3" s="17"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
+      <c r="B3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="4">
+        <v>100001</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C4" s="4">
-        <v>110033</v>
+        <v>100002</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
@@ -1593,13 +1657,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C5" s="4">
-        <v>110034</v>
+        <v>100003</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
@@ -1620,13 +1684,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C6" s="4">
-        <v>110031</v>
+        <v>100004</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -1647,13 +1711,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C7" s="4">
-        <v>110037</v>
+        <v>100007</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>159</v>
+        <v>67</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
@@ -1671,16 +1735,16 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>4</v>
+        <v>285</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>5</v>
+        <v>314</v>
       </c>
       <c r="C8" s="4">
-        <v>110005</v>
+        <v>100008</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>162</v>
+        <v>295</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
@@ -1701,13 +1765,13 @@
         <v>4</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C9" s="4">
-        <v>110038</v>
+        <v>100009</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
@@ -1728,13 +1792,13 @@
         <v>4</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C10" s="4">
-        <v>110007</v>
+        <v>100010</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>161</v>
+        <v>70</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
@@ -1755,13 +1819,13 @@
         <v>4</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C11" s="4">
-        <v>110008</v>
+        <v>100011</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>160</v>
+        <v>66</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
@@ -1782,13 +1846,13 @@
         <v>4</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C12" s="4">
-        <v>110012</v>
+        <v>100012</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>163</v>
+        <v>77</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
@@ -1809,13 +1873,13 @@
         <v>4</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C13" s="4">
-        <v>110040</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>164</v>
+        <v>100013</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
@@ -1836,13 +1900,13 @@
         <v>4</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C14" s="4">
-        <v>110021</v>
+        <v>100014</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
@@ -1863,13 +1927,13 @@
         <v>4</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C15" s="4">
-        <v>110035</v>
+        <v>100015</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
@@ -1890,13 +1954,13 @@
         <v>4</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C16" s="4">
-        <v>110014</v>
+        <v>100016</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
@@ -1917,13 +1981,13 @@
         <v>4</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C17" s="4">
-        <v>110016</v>
+        <v>100017</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
@@ -1941,16 +2005,16 @@
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>4</v>
+        <v>285</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>5</v>
+        <v>313</v>
       </c>
       <c r="C18" s="4">
-        <v>110018</v>
+        <v>110001</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>57</v>
+        <v>296</v>
       </c>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
@@ -1974,10 +2038,10 @@
         <v>5</v>
       </c>
       <c r="C19" s="4">
-        <v>110023</v>
+        <v>110005</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>58</v>
+        <v>162</v>
       </c>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
@@ -2001,10 +2065,10 @@
         <v>5</v>
       </c>
       <c r="C20" s="4">
-        <v>110025</v>
+        <v>110007</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>59</v>
+        <v>161</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
@@ -2028,10 +2092,10 @@
         <v>5</v>
       </c>
       <c r="C21" s="4">
-        <v>110026</v>
+        <v>110008</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -2055,10 +2119,10 @@
         <v>5</v>
       </c>
       <c r="C22" s="4">
-        <v>110027</v>
+        <v>110012</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>60</v>
+        <v>163</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
@@ -2082,10 +2146,10 @@
         <v>5</v>
       </c>
       <c r="C23" s="4">
-        <v>110030</v>
+        <v>110014</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
@@ -2106,13 +2170,13 @@
         <v>4</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C24" s="4">
-        <v>100004</v>
+        <v>110016</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="E24" s="6"/>
       <c r="F24" s="6"/>
@@ -2133,13 +2197,13 @@
         <v>4</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C25" s="4">
-        <v>100017</v>
+        <v>110018</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
@@ -2160,13 +2224,13 @@
         <v>4</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C26" s="4">
-        <v>100013</v>
+        <v>110021</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="E26" s="6"/>
       <c r="F26" s="6"/>
@@ -2187,13 +2251,13 @@
         <v>4</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C27" s="4">
-        <v>100012</v>
+        <v>110023</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="6"/>
@@ -2214,13 +2278,13 @@
         <v>4</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C28" s="4">
-        <v>100002</v>
+        <v>110025</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
@@ -2241,13 +2305,13 @@
         <v>4</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C29" s="4">
-        <v>100015</v>
+        <v>110026</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>65</v>
+        <v>158</v>
       </c>
       <c r="E29" s="6"/>
       <c r="F29" s="6"/>
@@ -2268,13 +2332,13 @@
         <v>4</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C30" s="4">
-        <v>100011</v>
+        <v>110027</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
@@ -2295,13 +2359,13 @@
         <v>4</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C31" s="4">
-        <v>100007</v>
+        <v>110030</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
@@ -2322,13 +2386,13 @@
         <v>4</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C32" s="4">
-        <v>100001</v>
+        <v>110031</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
@@ -2349,13 +2413,13 @@
         <v>4</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C33" s="4">
-        <v>100014</v>
+        <v>110033</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
@@ -2376,13 +2440,13 @@
         <v>4</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C34" s="4">
-        <v>100010</v>
+        <v>110034</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
@@ -2403,13 +2467,13 @@
         <v>4</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C35" s="4">
-        <v>100003</v>
+        <v>110035</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
@@ -2430,13 +2494,13 @@
         <v>4</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C36" s="4">
-        <v>100016</v>
+        <v>110036</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
@@ -2457,13 +2521,13 @@
         <v>4</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C37" s="4">
-        <v>100009</v>
+        <v>110037</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>73</v>
+        <v>159</v>
       </c>
       <c r="E37" s="6"/>
       <c r="F37" s="6"/>
@@ -2484,13 +2548,13 @@
         <v>4</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>78</v>
+        <v>5</v>
+      </c>
+      <c r="C38" s="4">
+        <v>110038</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
@@ -2511,13 +2575,13 @@
         <v>4</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>80</v>
+        <v>5</v>
+      </c>
+      <c r="C39" s="4">
+        <v>110040</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>81</v>
+        <v>164</v>
       </c>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
@@ -2535,16 +2599,16 @@
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>4</v>
+        <v>316</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>82</v>
+        <v>11</v>
+      </c>
+      <c r="C40" s="4">
+        <v>200001</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E40" s="6"/>
       <c r="F40" s="6"/>
@@ -2562,16 +2626,16 @@
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>4</v>
+        <v>316</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>84</v>
+        <v>11</v>
+      </c>
+      <c r="C41" s="4">
+        <v>200002</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
@@ -2589,16 +2653,16 @@
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>4</v>
+        <v>316</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>86</v>
+        <v>11</v>
+      </c>
+      <c r="C42" s="4">
+        <v>200003</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
@@ -2616,16 +2680,16 @@
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>4</v>
+        <v>316</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>88</v>
+        <v>11</v>
+      </c>
+      <c r="C43" s="4">
+        <v>200004</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
@@ -2643,16 +2707,16 @@
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>4</v>
+        <v>316</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>62</v>
+        <v>11</v>
+      </c>
+      <c r="C44" s="4">
+        <v>200005</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
@@ -2670,16 +2734,16 @@
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>14</v>
+        <v>316</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C45" s="4">
-        <v>500025</v>
+        <v>200006</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E45" s="6"/>
       <c r="F45" s="6"/>
@@ -2697,16 +2761,16 @@
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>14</v>
+        <v>316</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C46" s="4">
-        <v>500020</v>
+        <v>200007</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E46" s="6"/>
       <c r="F46" s="6"/>
@@ -2724,16 +2788,16 @@
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>14</v>
+        <v>316</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C47" s="4">
-        <v>500021</v>
+        <v>200008</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
@@ -2751,16 +2815,16 @@
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>16</v>
+        <v>315</v>
       </c>
       <c r="C48" s="4">
-        <v>500019</v>
+        <v>300001</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>102</v>
+        <v>297</v>
       </c>
       <c r="E48" s="6"/>
       <c r="F48" s="6"/>
@@ -2778,16 +2842,16 @@
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C49" s="4">
-        <v>500012</v>
+        <v>300002</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="E49" s="6"/>
       <c r="F49" s="6"/>
@@ -2805,16 +2869,16 @@
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C50" s="4">
-        <v>500004</v>
+        <v>300003</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>104</v>
+        <v>298</v>
       </c>
       <c r="E50" s="6"/>
       <c r="F50" s="6"/>
@@ -2832,16 +2896,16 @@
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C51" s="4">
-        <v>500014</v>
+        <v>400000</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
@@ -2859,16 +2923,16 @@
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>14</v>
+        <v>286</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="C52" s="4">
-        <v>500027</v>
+        <v>400001</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>165</v>
+        <v>116</v>
       </c>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
@@ -2886,32 +2950,24 @@
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="C53" s="4">
-        <v>600008</v>
+        <v>400002</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="E53" s="6"/>
-      <c r="F53" s="12" t="s">
-        <v>280</v>
-      </c>
-      <c r="G53" s="12" t="s">
-        <v>281</v>
-      </c>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
       <c r="H53" s="6"/>
       <c r="I53" s="6"/>
-      <c r="J53" s="12" t="s">
-        <v>282</v>
-      </c>
-      <c r="K53" s="12" t="s">
-        <v>283</v>
-      </c>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
       <c r="L53" s="6"/>
       <c r="M53" s="6"/>
       <c r="N53" s="6"/>
@@ -2921,32 +2977,24 @@
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>19</v>
+        <v>286</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C54" s="4">
-        <v>600011</v>
+        <v>400003</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E54" s="6"/>
-      <c r="F54" s="12" t="s">
-        <v>280</v>
-      </c>
-      <c r="G54" s="12" t="s">
-        <v>281</v>
-      </c>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
       <c r="H54" s="6"/>
       <c r="I54" s="6"/>
-      <c r="J54" s="12" t="s">
-        <v>282</v>
-      </c>
-      <c r="K54" s="12" t="s">
-        <v>283</v>
-      </c>
+      <c r="J54" s="6"/>
+      <c r="K54" s="6"/>
       <c r="L54" s="6"/>
       <c r="M54" s="6"/>
       <c r="N54" s="6"/>
@@ -2956,16 +3004,14 @@
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>23</v>
-      </c>
+        <v>286</v>
+      </c>
+      <c r="B55" s="4"/>
       <c r="C55" s="4">
-        <v>600007</v>
+        <v>400004</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>110</v>
+        <v>258</v>
       </c>
       <c r="E55" s="6"/>
       <c r="F55" s="6"/>
@@ -2983,20 +3029,16 @@
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>24</v>
-      </c>
+        <v>286</v>
+      </c>
+      <c r="B56" s="4"/>
       <c r="C56" s="4">
-        <v>600006</v>
+        <v>400007</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="E56" s="12" t="s">
-        <v>264</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="E56" s="6"/>
       <c r="F56" s="6"/>
       <c r="G56" s="6"/>
       <c r="H56" s="6"/>
@@ -3012,24 +3054,20 @@
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>19</v>
+        <v>317</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>25</v>
+        <v>318</v>
       </c>
       <c r="C57" s="4">
-        <v>600005</v>
+        <v>400009</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>112</v>
+        <v>299</v>
       </c>
       <c r="E57" s="6"/>
-      <c r="F57" s="12" t="s">
-        <v>265</v>
-      </c>
-      <c r="G57" s="12" t="s">
-        <v>266</v>
-      </c>
+      <c r="F57" s="6"/>
+      <c r="G57" s="6"/>
       <c r="H57" s="6"/>
       <c r="I57" s="6"/>
       <c r="J57" s="6"/>
@@ -3043,32 +3081,24 @@
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>19</v>
+        <v>317</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>26</v>
+        <v>318</v>
       </c>
       <c r="C58" s="4">
-        <v>600002</v>
+        <v>400011</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>113</v>
+        <v>300</v>
       </c>
       <c r="E58" s="6"/>
-      <c r="F58" s="12" t="s">
-        <v>280</v>
-      </c>
-      <c r="G58" s="12" t="s">
-        <v>281</v>
-      </c>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
       <c r="H58" s="6"/>
       <c r="I58" s="6"/>
-      <c r="J58" s="12" t="s">
-        <v>282</v>
-      </c>
-      <c r="K58" s="12" t="s">
-        <v>283</v>
-      </c>
+      <c r="J58" s="6"/>
+      <c r="K58" s="6"/>
       <c r="L58" s="6"/>
       <c r="M58" s="6"/>
       <c r="N58" s="6"/>
@@ -3078,32 +3108,22 @@
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>28</v>
-      </c>
+        <v>286</v>
+      </c>
+      <c r="B59" s="4"/>
       <c r="C59" s="4">
-        <v>600009</v>
+        <v>400012</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E59" s="6"/>
-      <c r="F59" s="12" t="s">
-        <v>280</v>
-      </c>
-      <c r="G59" s="12" t="s">
-        <v>281</v>
-      </c>
+      <c r="F59" s="6"/>
+      <c r="G59" s="6"/>
       <c r="H59" s="6"/>
       <c r="I59" s="6"/>
-      <c r="J59" s="12" t="s">
-        <v>282</v>
-      </c>
-      <c r="K59" s="12" t="s">
-        <v>283</v>
-      </c>
+      <c r="J59" s="6"/>
+      <c r="K59" s="6"/>
       <c r="L59" s="6"/>
       <c r="M59" s="6"/>
       <c r="N59" s="6"/>
@@ -3113,16 +3133,16 @@
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="C60" s="4">
-        <v>600004</v>
+        <v>400013</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E60" s="6"/>
       <c r="F60" s="6"/>
@@ -3140,16 +3160,16 @@
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C61" s="4">
-        <v>600003</v>
+        <v>400014</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="E61" s="6"/>
       <c r="F61" s="6"/>
@@ -3167,21 +3187,19 @@
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>27</v>
+        <v>319</v>
       </c>
       <c r="C62" s="4">
-        <v>600001</v>
+        <v>500003</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>114</v>
+        <v>301</v>
       </c>
       <c r="E62" s="6"/>
-      <c r="F62" s="19" t="s">
-        <v>284</v>
-      </c>
+      <c r="F62" s="6"/>
       <c r="G62" s="6"/>
       <c r="H62" s="6"/>
       <c r="I62" s="6"/>
@@ -3196,16 +3214,16 @@
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="C63" s="4">
-        <v>700015</v>
+        <v>500004</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>124</v>
+        <v>104</v>
       </c>
       <c r="E63" s="6"/>
       <c r="F63" s="6"/>
@@ -3223,16 +3241,16 @@
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>36</v>
+        <v>319</v>
       </c>
       <c r="C64" s="4">
-        <v>700014</v>
+        <v>500009</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>125</v>
+        <v>302</v>
       </c>
       <c r="E64" s="6"/>
       <c r="F64" s="6"/>
@@ -3250,16 +3268,16 @@
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
-        <v>35</v>
+        <v>287</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>36</v>
+        <v>288</v>
       </c>
       <c r="C65" s="4">
-        <v>700013</v>
+        <v>500010</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>126</v>
+        <v>303</v>
       </c>
       <c r="E65" s="6"/>
       <c r="F65" s="6"/>
@@ -3277,16 +3295,16 @@
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
-        <v>35</v>
+        <v>287</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>36</v>
+        <v>288</v>
       </c>
       <c r="C66" s="4">
-        <v>700016</v>
+        <v>500011</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>127</v>
+        <v>304</v>
       </c>
       <c r="E66" s="6"/>
       <c r="F66" s="6"/>
@@ -3304,16 +3322,16 @@
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="C67" s="4">
-        <v>700007</v>
+        <v>500012</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="E67" s="6"/>
       <c r="F67" s="6"/>
@@ -3331,16 +3349,16 @@
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
-        <v>35</v>
+        <v>287</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>37</v>
+        <v>288</v>
       </c>
       <c r="C68" s="4">
-        <v>700005</v>
+        <v>500013</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>129</v>
+        <v>305</v>
       </c>
       <c r="E68" s="6"/>
       <c r="F68" s="6"/>
@@ -3358,16 +3376,16 @@
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="C69" s="4">
-        <v>700008</v>
+        <v>500014</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>130</v>
+        <v>105</v>
       </c>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
@@ -3385,16 +3403,16 @@
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
-        <v>35</v>
+        <v>287</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>37</v>
+        <v>288</v>
       </c>
       <c r="C70" s="4">
-        <v>700006</v>
+        <v>500018</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>131</v>
+        <v>306</v>
       </c>
       <c r="E70" s="6"/>
       <c r="F70" s="6"/>
@@ -3412,16 +3430,16 @@
     </row>
     <row r="71" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C71" s="4">
-        <v>700002</v>
+        <v>500019</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>132</v>
+        <v>102</v>
       </c>
       <c r="E71" s="6"/>
       <c r="F71" s="6"/>
@@ -3439,16 +3457,16 @@
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C72" s="4">
-        <v>700004</v>
+        <v>500020</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>133</v>
+        <v>100</v>
       </c>
       <c r="E72" s="6"/>
       <c r="F72" s="6"/>
@@ -3466,16 +3484,16 @@
     </row>
     <row r="73" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C73" s="4">
-        <v>700003</v>
+        <v>500021</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>134</v>
+        <v>101</v>
       </c>
       <c r="E73" s="6"/>
       <c r="F73" s="6"/>
@@ -3493,16 +3511,16 @@
     </row>
     <row r="74" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="C74" s="4">
-        <v>700001</v>
+        <v>500025</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>135</v>
+        <v>99</v>
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="6"/>
@@ -3520,16 +3538,16 @@
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
-        <v>35</v>
+        <v>287</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>39</v>
+        <v>288</v>
       </c>
       <c r="C75" s="4">
-        <v>700019</v>
+        <v>500026</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>136</v>
+        <v>307</v>
       </c>
       <c r="E75" s="6"/>
       <c r="F75" s="6"/>
@@ -3547,16 +3565,16 @@
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="C76" s="4">
-        <v>700018</v>
+        <v>500027</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>137</v>
+        <v>165</v>
       </c>
       <c r="E76" s="6"/>
       <c r="F76" s="6"/>
@@ -3574,19 +3592,21 @@
     </row>
     <row r="77" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="C77" s="4">
-        <v>700017</v>
+        <v>600001</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="E77" s="6"/>
-      <c r="F77" s="6"/>
+      <c r="F77" s="6" t="s">
+        <v>284</v>
+      </c>
       <c r="G77" s="6"/>
       <c r="H77" s="6"/>
       <c r="I77" s="6"/>
@@ -3601,24 +3621,32 @@
     </row>
     <row r="78" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="C78" s="4">
-        <v>700020</v>
+        <v>600002</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>139</v>
+        <v>113</v>
       </c>
       <c r="E78" s="6"/>
-      <c r="F78" s="6"/>
-      <c r="G78" s="6"/>
+      <c r="F78" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="G78" s="6" t="s">
+        <v>281</v>
+      </c>
       <c r="H78" s="6"/>
       <c r="I78" s="6"/>
-      <c r="J78" s="6"/>
-      <c r="K78" s="6"/>
+      <c r="J78" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="K78" s="6" t="s">
+        <v>283</v>
+      </c>
       <c r="L78" s="6"/>
       <c r="M78" s="6"/>
       <c r="N78" s="6"/>
@@ -3628,16 +3656,16 @@
     </row>
     <row r="79" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="C79" s="4">
-        <v>700023</v>
+        <v>600003</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>140</v>
+        <v>109</v>
       </c>
       <c r="E79" s="6"/>
       <c r="F79" s="6"/>
@@ -3655,16 +3683,16 @@
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="C80" s="4">
-        <v>700022</v>
+        <v>600004</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>141</v>
+        <v>108</v>
       </c>
       <c r="E80" s="6"/>
       <c r="F80" s="6"/>
@@ -3682,20 +3710,24 @@
     </row>
     <row r="81" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="C81" s="4">
-        <v>700021</v>
+        <v>600005</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="E81" s="6"/>
-      <c r="F81" s="6"/>
-      <c r="G81" s="6"/>
+      <c r="F81" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="G81" s="6" t="s">
+        <v>266</v>
+      </c>
       <c r="H81" s="6"/>
       <c r="I81" s="6"/>
       <c r="J81" s="6"/>
@@ -3709,18 +3741,20 @@
     </row>
     <row r="82" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="C82" s="4">
-        <v>700024</v>
+        <v>600006</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="E82" s="6"/>
+        <v>111</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>264</v>
+      </c>
       <c r="F82" s="6"/>
       <c r="G82" s="6"/>
       <c r="H82" s="6"/>
@@ -3736,16 +3770,16 @@
     </row>
     <row r="83" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="C83" s="4">
-        <v>900006</v>
+        <v>600007</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>147</v>
+        <v>110</v>
       </c>
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
@@ -3763,24 +3797,32 @@
     </row>
     <row r="84" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="C84" s="4">
-        <v>900002</v>
+        <v>600008</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>149</v>
+        <v>106</v>
       </c>
       <c r="E84" s="6"/>
-      <c r="F84" s="6"/>
-      <c r="G84" s="6"/>
+      <c r="F84" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="G84" s="6" t="s">
+        <v>281</v>
+      </c>
       <c r="H84" s="6"/>
       <c r="I84" s="6"/>
-      <c r="J84" s="6"/>
-      <c r="K84" s="6"/>
+      <c r="J84" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="K84" s="6" t="s">
+        <v>283</v>
+      </c>
       <c r="L84" s="6"/>
       <c r="M84" s="6"/>
       <c r="N84" s="6"/>
@@ -3790,33 +3832,31 @@
     </row>
     <row r="85" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="C85" s="4">
-        <v>900003</v>
+        <v>600009</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="E85" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="F85" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="G85" s="13" t="s">
-        <v>269</v>
+        <v>115</v>
+      </c>
+      <c r="E85" s="6"/>
+      <c r="F85" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="G85" s="6" t="s">
+        <v>281</v>
       </c>
       <c r="H85" s="6"/>
       <c r="I85" s="6"/>
-      <c r="J85" s="14" t="s">
-        <v>274</v>
-      </c>
-      <c r="K85" s="14" t="s">
-        <v>275</v>
+      <c r="J85" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="K85" s="6" t="s">
+        <v>283</v>
       </c>
       <c r="L85" s="6"/>
       <c r="M85" s="6"/>
@@ -3827,34 +3867,22 @@
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B86" s="4" t="s">
-        <v>47</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="B86" s="4"/>
       <c r="C86" s="4">
-        <v>900000</v>
+        <v>600010</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="E86" s="13" t="s">
-        <v>272</v>
-      </c>
-      <c r="F86" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="G86" s="13" t="s">
-        <v>269</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="E86" s="6"/>
+      <c r="F86" s="6"/>
+      <c r="G86" s="6"/>
       <c r="H86" s="6"/>
       <c r="I86" s="6"/>
-      <c r="J86" s="14" t="s">
-        <v>274</v>
-      </c>
-      <c r="K86" s="14" t="s">
-        <v>275</v>
-      </c>
+      <c r="J86" s="6"/>
+      <c r="K86" s="6"/>
       <c r="L86" s="6"/>
       <c r="M86" s="6"/>
       <c r="N86" s="6"/>
@@ -3864,33 +3892,31 @@
     </row>
     <row r="87" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="C87" s="4">
-        <v>900001</v>
+        <v>600011</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="E87" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="F87" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="G87" s="13" t="s">
-        <v>269</v>
+        <v>107</v>
+      </c>
+      <c r="E87" s="6"/>
+      <c r="F87" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="G87" s="6" t="s">
+        <v>281</v>
       </c>
       <c r="H87" s="6"/>
       <c r="I87" s="6"/>
-      <c r="J87" s="14" t="s">
-        <v>274</v>
-      </c>
-      <c r="K87" s="14" t="s">
-        <v>275</v>
+      <c r="J87" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="K87" s="6" t="s">
+        <v>283</v>
       </c>
       <c r="L87" s="6"/>
       <c r="M87" s="6"/>
@@ -3901,16 +3927,14 @@
     </row>
     <row r="88" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B88" s="4" t="s">
-        <v>41</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="B88" s="4"/>
       <c r="C88" s="4">
-        <v>900004</v>
+        <v>600012</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="E88" s="6"/>
       <c r="F88" s="6"/>
@@ -3928,16 +3952,16 @@
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C89" s="4">
-        <v>900005</v>
+        <v>700001</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="E89" s="6"/>
       <c r="F89" s="6"/>
@@ -3955,16 +3979,16 @@
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C90" s="4">
-        <v>900007</v>
+        <v>700002</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="E90" s="6"/>
       <c r="F90" s="6"/>
@@ -3982,16 +4006,16 @@
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C91" s="4">
-        <v>900008</v>
+        <v>700003</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="E91" s="6"/>
       <c r="F91" s="6"/>
@@ -4009,16 +4033,16 @@
     </row>
     <row r="92" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C92" s="4">
-        <v>900009</v>
+        <v>700004</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="E92" s="6"/>
       <c r="F92" s="6"/>
@@ -4034,7 +4058,1064 @@
       <c r="P92" s="6"/>
       <c r="Q92" s="6"/>
     </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A93" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C93" s="4">
+        <v>700005</v>
+      </c>
+      <c r="D93" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E93" s="6"/>
+      <c r="F93" s="6"/>
+      <c r="G93" s="6"/>
+      <c r="H93" s="6"/>
+      <c r="I93" s="6"/>
+      <c r="J93" s="6"/>
+      <c r="K93" s="6"/>
+      <c r="L93" s="6"/>
+      <c r="M93" s="6"/>
+      <c r="N93" s="6"/>
+      <c r="O93" s="6"/>
+      <c r="P93" s="6"/>
+      <c r="Q93" s="6"/>
+    </row>
+    <row r="94" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A94" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C94" s="4">
+        <v>700006</v>
+      </c>
+      <c r="D94" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="E94" s="6"/>
+      <c r="F94" s="6"/>
+      <c r="G94" s="6"/>
+      <c r="H94" s="6"/>
+      <c r="I94" s="6"/>
+      <c r="J94" s="6"/>
+      <c r="K94" s="6"/>
+      <c r="L94" s="6"/>
+      <c r="M94" s="6"/>
+      <c r="N94" s="6"/>
+      <c r="O94" s="6"/>
+      <c r="P94" s="6"/>
+      <c r="Q94" s="6"/>
+    </row>
+    <row r="95" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A95" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C95" s="4">
+        <v>700007</v>
+      </c>
+      <c r="D95" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="E95" s="6"/>
+      <c r="F95" s="6"/>
+      <c r="G95" s="6"/>
+      <c r="H95" s="6"/>
+      <c r="I95" s="6"/>
+      <c r="J95" s="6"/>
+      <c r="K95" s="6"/>
+      <c r="L95" s="6"/>
+      <c r="M95" s="6"/>
+      <c r="N95" s="6"/>
+      <c r="O95" s="6"/>
+      <c r="P95" s="6"/>
+      <c r="Q95" s="6"/>
+    </row>
+    <row r="96" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A96" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C96" s="4">
+        <v>700008</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E96" s="6"/>
+      <c r="F96" s="6"/>
+      <c r="G96" s="6"/>
+      <c r="H96" s="6"/>
+      <c r="I96" s="6"/>
+      <c r="J96" s="6"/>
+      <c r="K96" s="6"/>
+      <c r="L96" s="6"/>
+      <c r="M96" s="6"/>
+      <c r="N96" s="6"/>
+      <c r="O96" s="6"/>
+      <c r="P96" s="6"/>
+      <c r="Q96" s="6"/>
+    </row>
+    <row r="97" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A97" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C97" s="4">
+        <v>700009</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="E97" s="6"/>
+      <c r="F97" s="6"/>
+      <c r="G97" s="6"/>
+      <c r="H97" s="6"/>
+      <c r="I97" s="6"/>
+      <c r="J97" s="6"/>
+      <c r="K97" s="6"/>
+      <c r="L97" s="6"/>
+      <c r="M97" s="6"/>
+      <c r="N97" s="6"/>
+      <c r="O97" s="6"/>
+      <c r="P97" s="6"/>
+      <c r="Q97" s="6"/>
+    </row>
+    <row r="98" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A98" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="C98" s="4">
+        <v>700010</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="E98" s="6"/>
+      <c r="F98" s="6"/>
+      <c r="G98" s="6"/>
+      <c r="H98" s="6"/>
+      <c r="I98" s="6"/>
+      <c r="J98" s="6"/>
+      <c r="K98" s="6"/>
+      <c r="L98" s="6"/>
+      <c r="M98" s="6"/>
+      <c r="N98" s="6"/>
+      <c r="O98" s="6"/>
+      <c r="P98" s="6"/>
+      <c r="Q98" s="6"/>
+    </row>
+    <row r="99" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A99" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="C99" s="4">
+        <v>700011</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="E99" s="6"/>
+      <c r="F99" s="6"/>
+      <c r="G99" s="6"/>
+      <c r="H99" s="6"/>
+      <c r="I99" s="6"/>
+      <c r="J99" s="6"/>
+      <c r="K99" s="6"/>
+      <c r="L99" s="6"/>
+      <c r="M99" s="6"/>
+      <c r="N99" s="6"/>
+      <c r="O99" s="6"/>
+      <c r="P99" s="6"/>
+      <c r="Q99" s="6"/>
+    </row>
+    <row r="100" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A100" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="C100" s="4">
+        <v>700012</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="E100" s="6"/>
+      <c r="F100" s="6"/>
+      <c r="G100" s="6"/>
+      <c r="H100" s="6"/>
+      <c r="I100" s="6"/>
+      <c r="J100" s="6"/>
+      <c r="K100" s="6"/>
+      <c r="L100" s="6"/>
+      <c r="M100" s="6"/>
+      <c r="N100" s="6"/>
+      <c r="O100" s="6"/>
+      <c r="P100" s="6"/>
+      <c r="Q100" s="6"/>
+    </row>
+    <row r="101" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A101" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C101" s="4">
+        <v>700013</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E101" s="6"/>
+      <c r="F101" s="6"/>
+      <c r="G101" s="6"/>
+      <c r="H101" s="6"/>
+      <c r="I101" s="6"/>
+      <c r="J101" s="6"/>
+      <c r="K101" s="6"/>
+      <c r="L101" s="6"/>
+      <c r="M101" s="6"/>
+      <c r="N101" s="6"/>
+      <c r="O101" s="6"/>
+      <c r="P101" s="6"/>
+      <c r="Q101" s="6"/>
+    </row>
+    <row r="102" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A102" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C102" s="4">
+        <v>700014</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E102" s="6"/>
+      <c r="F102" s="6"/>
+      <c r="G102" s="6"/>
+      <c r="H102" s="6"/>
+      <c r="I102" s="6"/>
+      <c r="J102" s="6"/>
+      <c r="K102" s="6"/>
+      <c r="L102" s="6"/>
+      <c r="M102" s="6"/>
+      <c r="N102" s="6"/>
+      <c r="O102" s="6"/>
+      <c r="P102" s="6"/>
+      <c r="Q102" s="6"/>
+    </row>
+    <row r="103" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A103" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C103" s="4">
+        <v>700015</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E103" s="6"/>
+      <c r="F103" s="6"/>
+      <c r="G103" s="6"/>
+      <c r="H103" s="6"/>
+      <c r="I103" s="6"/>
+      <c r="J103" s="6"/>
+      <c r="K103" s="6"/>
+      <c r="L103" s="6"/>
+      <c r="M103" s="6"/>
+      <c r="N103" s="6"/>
+      <c r="O103" s="6"/>
+      <c r="P103" s="6"/>
+      <c r="Q103" s="6"/>
+    </row>
+    <row r="104" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A104" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C104" s="4">
+        <v>700016</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E104" s="6"/>
+      <c r="F104" s="6"/>
+      <c r="G104" s="6"/>
+      <c r="H104" s="6"/>
+      <c r="I104" s="6"/>
+      <c r="J104" s="6"/>
+      <c r="K104" s="6"/>
+      <c r="L104" s="6"/>
+      <c r="M104" s="6"/>
+      <c r="N104" s="6"/>
+      <c r="O104" s="6"/>
+      <c r="P104" s="6"/>
+      <c r="Q104" s="6"/>
+    </row>
+    <row r="105" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A105" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C105" s="4">
+        <v>700017</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="E105" s="6"/>
+      <c r="F105" s="6"/>
+      <c r="G105" s="6"/>
+      <c r="H105" s="6"/>
+      <c r="I105" s="6"/>
+      <c r="J105" s="6"/>
+      <c r="K105" s="6"/>
+      <c r="L105" s="6"/>
+      <c r="M105" s="6"/>
+      <c r="N105" s="6"/>
+      <c r="O105" s="6"/>
+      <c r="P105" s="6"/>
+      <c r="Q105" s="6"/>
+    </row>
+    <row r="106" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A106" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C106" s="4">
+        <v>700018</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E106" s="6"/>
+      <c r="F106" s="6"/>
+      <c r="G106" s="6"/>
+      <c r="H106" s="6"/>
+      <c r="I106" s="6"/>
+      <c r="J106" s="6"/>
+      <c r="K106" s="6"/>
+      <c r="L106" s="6"/>
+      <c r="M106" s="6"/>
+      <c r="N106" s="6"/>
+      <c r="O106" s="6"/>
+      <c r="P106" s="6"/>
+      <c r="Q106" s="6"/>
+    </row>
+    <row r="107" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A107" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C107" s="4">
+        <v>700019</v>
+      </c>
+      <c r="D107" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E107" s="6"/>
+      <c r="F107" s="6"/>
+      <c r="G107" s="6"/>
+      <c r="H107" s="6"/>
+      <c r="I107" s="6"/>
+      <c r="J107" s="6"/>
+      <c r="K107" s="6"/>
+      <c r="L107" s="6"/>
+      <c r="M107" s="6"/>
+      <c r="N107" s="6"/>
+      <c r="O107" s="6"/>
+      <c r="P107" s="6"/>
+      <c r="Q107" s="6"/>
+    </row>
+    <row r="108" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A108" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C108" s="4">
+        <v>700020</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E108" s="6"/>
+      <c r="F108" s="6"/>
+      <c r="G108" s="6"/>
+      <c r="H108" s="6"/>
+      <c r="I108" s="6"/>
+      <c r="J108" s="6"/>
+      <c r="K108" s="6"/>
+      <c r="L108" s="6"/>
+      <c r="M108" s="6"/>
+      <c r="N108" s="6"/>
+      <c r="O108" s="6"/>
+      <c r="P108" s="6"/>
+      <c r="Q108" s="6"/>
+    </row>
+    <row r="109" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A109" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C109" s="4">
+        <v>700021</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E109" s="6"/>
+      <c r="F109" s="6"/>
+      <c r="G109" s="6"/>
+      <c r="H109" s="6"/>
+      <c r="I109" s="6"/>
+      <c r="J109" s="6"/>
+      <c r="K109" s="6"/>
+      <c r="L109" s="6"/>
+      <c r="M109" s="6"/>
+      <c r="N109" s="6"/>
+      <c r="O109" s="6"/>
+      <c r="P109" s="6"/>
+      <c r="Q109" s="6"/>
+    </row>
+    <row r="110" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A110" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C110" s="4">
+        <v>700022</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E110" s="6"/>
+      <c r="F110" s="6"/>
+      <c r="G110" s="6"/>
+      <c r="H110" s="6"/>
+      <c r="I110" s="6"/>
+      <c r="J110" s="6"/>
+      <c r="K110" s="6"/>
+      <c r="L110" s="6"/>
+      <c r="M110" s="6"/>
+      <c r="N110" s="6"/>
+      <c r="O110" s="6"/>
+      <c r="P110" s="6"/>
+      <c r="Q110" s="6"/>
+    </row>
+    <row r="111" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A111" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C111" s="4">
+        <v>700023</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E111" s="6"/>
+      <c r="F111" s="6"/>
+      <c r="G111" s="6"/>
+      <c r="H111" s="6"/>
+      <c r="I111" s="6"/>
+      <c r="J111" s="6"/>
+      <c r="K111" s="6"/>
+      <c r="L111" s="6"/>
+      <c r="M111" s="6"/>
+      <c r="N111" s="6"/>
+      <c r="O111" s="6"/>
+      <c r="P111" s="6"/>
+      <c r="Q111" s="6"/>
+    </row>
+    <row r="112" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A112" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C112" s="4">
+        <v>700024</v>
+      </c>
+      <c r="D112" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E112" s="6"/>
+      <c r="F112" s="6"/>
+      <c r="G112" s="6"/>
+      <c r="H112" s="6"/>
+      <c r="I112" s="6"/>
+      <c r="J112" s="6"/>
+      <c r="K112" s="6"/>
+      <c r="L112" s="6"/>
+      <c r="M112" s="6"/>
+      <c r="N112" s="6"/>
+      <c r="O112" s="6"/>
+      <c r="P112" s="6"/>
+      <c r="Q112" s="6"/>
+    </row>
+    <row r="113" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A113" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C113" s="4">
+        <v>900000</v>
+      </c>
+      <c r="D113" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="E113" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="F113" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="G113" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="H113" s="6"/>
+      <c r="I113" s="6"/>
+      <c r="J113" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="K113" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L113" s="6"/>
+      <c r="M113" s="6"/>
+      <c r="N113" s="6"/>
+      <c r="O113" s="6"/>
+      <c r="P113" s="6"/>
+      <c r="Q113" s="6"/>
+    </row>
+    <row r="114" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A114" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C114" s="4">
+        <v>900001</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="E114" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="F114" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="G114" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="H114" s="6"/>
+      <c r="I114" s="6"/>
+      <c r="J114" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="K114" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L114" s="6"/>
+      <c r="M114" s="6"/>
+      <c r="N114" s="6"/>
+      <c r="O114" s="6"/>
+      <c r="P114" s="6"/>
+      <c r="Q114" s="6"/>
+    </row>
+    <row r="115" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A115" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C115" s="4">
+        <v>900002</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E115" s="6"/>
+      <c r="F115" s="6"/>
+      <c r="G115" s="6"/>
+      <c r="H115" s="6"/>
+      <c r="I115" s="6"/>
+      <c r="J115" s="6"/>
+      <c r="K115" s="6"/>
+      <c r="L115" s="6"/>
+      <c r="M115" s="6"/>
+      <c r="N115" s="6"/>
+      <c r="O115" s="6"/>
+      <c r="P115" s="6"/>
+      <c r="Q115" s="6"/>
+    </row>
+    <row r="116" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A116" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C116" s="4">
+        <v>900003</v>
+      </c>
+      <c r="D116" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E116" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="F116" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="G116" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="H116" s="6"/>
+      <c r="I116" s="6"/>
+      <c r="J116" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="K116" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L116" s="6"/>
+      <c r="M116" s="6"/>
+      <c r="N116" s="6"/>
+      <c r="O116" s="6"/>
+      <c r="P116" s="6"/>
+      <c r="Q116" s="6"/>
+    </row>
+    <row r="117" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A117" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C117" s="4">
+        <v>900004</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E117" s="6"/>
+      <c r="F117" s="6"/>
+      <c r="G117" s="6"/>
+      <c r="H117" s="6"/>
+      <c r="I117" s="6"/>
+      <c r="J117" s="6"/>
+      <c r="K117" s="6"/>
+      <c r="L117" s="6"/>
+      <c r="M117" s="6"/>
+      <c r="N117" s="6"/>
+      <c r="O117" s="6"/>
+      <c r="P117" s="6"/>
+      <c r="Q117" s="6"/>
+    </row>
+    <row r="118" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A118" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C118" s="4">
+        <v>900005</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E118" s="6"/>
+      <c r="F118" s="6"/>
+      <c r="G118" s="6"/>
+      <c r="H118" s="6"/>
+      <c r="I118" s="6"/>
+      <c r="J118" s="6"/>
+      <c r="K118" s="6"/>
+      <c r="L118" s="6"/>
+      <c r="M118" s="6"/>
+      <c r="N118" s="6"/>
+      <c r="O118" s="6"/>
+      <c r="P118" s="6"/>
+      <c r="Q118" s="6"/>
+    </row>
+    <row r="119" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A119" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C119" s="4">
+        <v>900006</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="E119" s="6"/>
+      <c r="F119" s="6"/>
+      <c r="G119" s="6"/>
+      <c r="H119" s="6"/>
+      <c r="I119" s="6"/>
+      <c r="J119" s="6"/>
+      <c r="K119" s="6"/>
+      <c r="L119" s="6"/>
+      <c r="M119" s="6"/>
+      <c r="N119" s="6"/>
+      <c r="O119" s="6"/>
+      <c r="P119" s="6"/>
+      <c r="Q119" s="6"/>
+    </row>
+    <row r="120" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A120" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C120" s="4">
+        <v>900007</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E120" s="6"/>
+      <c r="F120" s="6"/>
+      <c r="G120" s="6"/>
+      <c r="H120" s="6"/>
+      <c r="I120" s="6"/>
+      <c r="J120" s="6"/>
+      <c r="K120" s="6"/>
+      <c r="L120" s="6"/>
+      <c r="M120" s="6"/>
+      <c r="N120" s="6"/>
+      <c r="O120" s="6"/>
+      <c r="P120" s="6"/>
+      <c r="Q120" s="6"/>
+    </row>
+    <row r="121" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A121" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C121" s="4">
+        <v>900008</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="E121" s="6"/>
+      <c r="F121" s="6"/>
+      <c r="G121" s="6"/>
+      <c r="H121" s="6"/>
+      <c r="I121" s="6"/>
+      <c r="J121" s="6"/>
+      <c r="K121" s="6"/>
+      <c r="L121" s="6"/>
+      <c r="M121" s="6"/>
+      <c r="N121" s="6"/>
+      <c r="O121" s="6"/>
+      <c r="P121" s="6"/>
+      <c r="Q121" s="6"/>
+    </row>
+    <row r="122" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A122" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C122" s="4">
+        <v>900009</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="E122" s="6"/>
+      <c r="F122" s="6"/>
+      <c r="G122" s="6"/>
+      <c r="H122" s="6"/>
+      <c r="I122" s="6"/>
+      <c r="J122" s="6"/>
+      <c r="K122" s="6"/>
+      <c r="L122" s="6"/>
+      <c r="M122" s="6"/>
+      <c r="N122" s="6"/>
+      <c r="O122" s="6"/>
+      <c r="P122" s="6"/>
+      <c r="Q122" s="6"/>
+    </row>
+    <row r="123" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A123" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="C123" s="4">
+        <v>900010</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="E123" s="6"/>
+      <c r="F123" s="6"/>
+      <c r="G123" s="6"/>
+      <c r="H123" s="6"/>
+      <c r="I123" s="6"/>
+      <c r="J123" s="6"/>
+      <c r="K123" s="6"/>
+      <c r="L123" s="6"/>
+      <c r="M123" s="6"/>
+      <c r="N123" s="6"/>
+      <c r="O123" s="6"/>
+      <c r="P123" s="6"/>
+      <c r="Q123" s="6"/>
+    </row>
+    <row r="124" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A124" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E124" s="6"/>
+      <c r="F124" s="6"/>
+      <c r="G124" s="6"/>
+      <c r="H124" s="6"/>
+      <c r="I124" s="6"/>
+      <c r="J124" s="6"/>
+      <c r="K124" s="6"/>
+      <c r="L124" s="6"/>
+      <c r="M124" s="6"/>
+      <c r="N124" s="6"/>
+      <c r="O124" s="6"/>
+      <c r="P124" s="6"/>
+      <c r="Q124" s="6"/>
+    </row>
+    <row r="125" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A125" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="E125" s="6"/>
+      <c r="F125" s="6"/>
+      <c r="G125" s="6"/>
+      <c r="H125" s="6"/>
+      <c r="I125" s="6"/>
+      <c r="J125" s="6"/>
+      <c r="K125" s="6"/>
+      <c r="L125" s="6"/>
+      <c r="M125" s="6"/>
+      <c r="N125" s="6"/>
+      <c r="O125" s="6"/>
+      <c r="P125" s="6"/>
+      <c r="Q125" s="6"/>
+    </row>
+    <row r="126" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A126" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E126" s="6"/>
+      <c r="F126" s="6"/>
+      <c r="G126" s="6"/>
+      <c r="H126" s="6"/>
+      <c r="I126" s="6"/>
+      <c r="J126" s="6"/>
+      <c r="K126" s="6"/>
+      <c r="L126" s="6"/>
+      <c r="M126" s="6"/>
+      <c r="N126" s="6"/>
+      <c r="O126" s="6"/>
+      <c r="P126" s="6"/>
+      <c r="Q126" s="6"/>
+    </row>
+    <row r="127" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A127" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E127" s="6"/>
+      <c r="F127" s="6"/>
+      <c r="G127" s="6"/>
+      <c r="H127" s="6"/>
+      <c r="I127" s="6"/>
+      <c r="J127" s="6"/>
+      <c r="K127" s="6"/>
+      <c r="L127" s="6"/>
+      <c r="M127" s="6"/>
+      <c r="N127" s="6"/>
+      <c r="O127" s="6"/>
+      <c r="P127" s="6"/>
+      <c r="Q127" s="6"/>
+    </row>
+    <row r="128" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A128" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E128" s="6"/>
+      <c r="F128" s="6"/>
+      <c r="G128" s="6"/>
+      <c r="H128" s="6"/>
+      <c r="I128" s="6"/>
+      <c r="J128" s="6"/>
+      <c r="K128" s="6"/>
+      <c r="L128" s="6"/>
+      <c r="M128" s="6"/>
+      <c r="N128" s="6"/>
+      <c r="O128" s="6"/>
+      <c r="P128" s="6"/>
+      <c r="Q128" s="6"/>
+    </row>
+    <row r="129" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A129" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E129" s="6"/>
+      <c r="F129" s="6"/>
+      <c r="G129" s="6"/>
+      <c r="H129" s="6"/>
+      <c r="I129" s="6"/>
+      <c r="J129" s="6"/>
+      <c r="K129" s="6"/>
+      <c r="L129" s="6"/>
+      <c r="M129" s="6"/>
+      <c r="N129" s="6"/>
+      <c r="O129" s="6"/>
+      <c r="P129" s="6"/>
+      <c r="Q129" s="6"/>
+    </row>
+    <row r="130" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A130" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E130" s="6"/>
+      <c r="F130" s="6"/>
+      <c r="G130" s="6"/>
+      <c r="H130" s="6"/>
+      <c r="I130" s="6"/>
+      <c r="J130" s="6"/>
+      <c r="K130" s="6"/>
+      <c r="L130" s="6"/>
+      <c r="M130" s="6"/>
+      <c r="N130" s="6"/>
+      <c r="O130" s="6"/>
+      <c r="P130" s="6"/>
+      <c r="Q130" s="6"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A2:Q130" xr:uid="{9157580D-EE50-43E2-A76D-B56C98A189DD}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v3.5: fix numpy/openpyxl corruption, checkbox de ingreso en Proyeccion
- Fix critico: numpy corrupto rompia openpyxl y dejaba vacios Salidas,
  Compras y descripciones de productos (Inventario). Se removio numpy
  (openpyxl no lo necesita) y se reconfirmo el pipeline completo.
- Nueva funcionalidad: tilde "ya ingreso" junto a Proyeccion abastecimiento
  en Proyeccion Produccion (solo visible en el mes en curso). Al tildar,
  excluye ese abastecimiento del calculo de saldo stock (ya esta reflejado
  en el stock en vivo), sin alterar venta real ni proyeccion mensual.
- Fix: los endpoints de guardado en caliente de Proyeccion leian el cache
  crudo (pre-overrides) en vez de los datos ya publicados, revirtiendo
  silenciosamente venta_actual/proyeccion_mensual del mes en curso en cada
  guardado. Ahora leen desde data_proyeccion.js publicado.
- Snapshot Versiones/v3.5/

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Productos/PRODUCTOS.xlsx
+++ b/Data/Productos/PRODUCTOS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SupplyDestileria\Documents\Bosque\Claude\Tablero operativo\Data\Productos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE60F89F-CA08-4A7A-B169-7497919C698E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8886B36E-854E-4BC2-A807-D99BE7A62969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{8FFC0A01-AC8B-4B89-A38C-E589AA3D5F39}"/>
   </bookViews>
@@ -18,28 +18,19 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">INSUMOS!$A$2:$Q$79</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PRODUCTOS!$A$2:$Q$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PRODUCTOS!$A$2:$Q$131</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="315">
   <si>
     <t>RUBRO</t>
   </si>
@@ -906,36 +897,15 @@
     <t>DECORMEC</t>
   </si>
   <si>
-    <t>Bebidas</t>
-  </si>
-  <si>
-    <t>Estuche</t>
-  </si>
-  <si>
-    <t>Combo</t>
-  </si>
-  <si>
     <t>Kit</t>
   </si>
   <si>
-    <t>Cristaleria</t>
-  </si>
-  <si>
-    <t>Indumentaria</t>
-  </si>
-  <si>
     <t>Gorro Lana</t>
   </si>
   <si>
     <t>Delantal</t>
   </si>
   <si>
-    <t>Mobiliario</t>
-  </si>
-  <si>
-    <t>Cartel</t>
-  </si>
-  <si>
     <t>GINTONIC BOSQUE LATA X 269 ML X 6 UN</t>
   </si>
   <si>
@@ -1009,6 +979,12 @@
   </si>
   <si>
     <t>LINEA CLASICA</t>
+  </si>
+  <si>
+    <t>BARRICA</t>
+  </si>
+  <si>
+    <t>BARRICA 225 LTS</t>
   </si>
 </sst>
 </file>
@@ -1226,9 +1202,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1266,7 +1242,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1372,7 +1348,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1514,7 +1490,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1522,7 +1498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9157580D-EE50-43E2-A76D-B56C98A189DD}">
-  <dimension ref="A1:Q130"/>
+  <dimension ref="A1:Q131"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -1545,7 +1521,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12.75" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:17" ht="36.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="24.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1735,16 +1711,16 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>285</v>
+        <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="C8" s="4">
         <v>100008</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
@@ -2005,16 +1981,16 @@
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>285</v>
+        <v>4</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="C18" s="4">
         <v>110001</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
@@ -2599,16 +2575,16 @@
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>316</v>
+        <v>4</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C40" s="4">
-        <v>200001</v>
+        <v>6</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>62</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="E40" s="6"/>
       <c r="F40" s="6"/>
@@ -2626,16 +2602,16 @@
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>316</v>
+        <v>4</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C41" s="4">
-        <v>200002</v>
+        <v>9</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>82</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
@@ -2653,16 +2629,16 @@
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>316</v>
+        <v>4</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C42" s="4">
-        <v>200003</v>
+        <v>9</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
@@ -2680,16 +2656,16 @@
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>316</v>
+        <v>4</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C43" s="4">
-        <v>200004</v>
+        <v>9</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>84</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
@@ -2707,16 +2683,16 @@
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>316</v>
+        <v>4</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C44" s="4">
-        <v>200005</v>
+        <v>9</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>80</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
@@ -2734,16 +2710,16 @@
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>316</v>
+        <v>4</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C45" s="4">
-        <v>200006</v>
+        <v>9</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>86</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E45" s="6"/>
       <c r="F45" s="6"/>
@@ -2761,16 +2737,16 @@
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>316</v>
+        <v>4</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C46" s="4">
-        <v>200007</v>
+        <v>9</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>88</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E46" s="6"/>
       <c r="F46" s="6"/>
@@ -2788,16 +2764,16 @@
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>11</v>
+        <v>311</v>
       </c>
       <c r="C47" s="4">
-        <v>200008</v>
+        <v>400009</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>93</v>
+        <v>292</v>
       </c>
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
@@ -2815,16 +2791,16 @@
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>33</v>
+        <v>310</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C48" s="4">
-        <v>300001</v>
+        <v>400011</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="E48" s="6"/>
       <c r="F48" s="6"/>
@@ -2842,16 +2818,16 @@
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>33</v>
+        <v>309</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="C49" s="4">
-        <v>300002</v>
+        <v>200001</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>123</v>
+        <v>91</v>
       </c>
       <c r="E49" s="6"/>
       <c r="F49" s="6"/>
@@ -2869,16 +2845,16 @@
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>33</v>
+        <v>309</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="C50" s="4">
-        <v>300003</v>
+        <v>200002</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>298</v>
+        <v>97</v>
       </c>
       <c r="E50" s="6"/>
       <c r="F50" s="6"/>
@@ -2896,16 +2872,16 @@
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>29</v>
+        <v>309</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="C51" s="4">
-        <v>400000</v>
+        <v>200003</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>121</v>
+        <v>90</v>
       </c>
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
@@ -2923,16 +2899,16 @@
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>286</v>
+        <v>309</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="C52" s="4">
-        <v>400001</v>
+        <v>200004</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
@@ -2950,16 +2926,16 @@
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>29</v>
+        <v>309</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="C53" s="4">
-        <v>400002</v>
+        <v>200005</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="E53" s="6"/>
       <c r="F53" s="6"/>
@@ -2977,16 +2953,16 @@
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>286</v>
+        <v>309</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="C54" s="4">
-        <v>400003</v>
+        <v>200006</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="E54" s="6"/>
       <c r="F54" s="6"/>
@@ -3004,14 +2980,16 @@
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>286</v>
-      </c>
-      <c r="B55" s="4"/>
+        <v>309</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="C55" s="4">
-        <v>400004</v>
+        <v>200007</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>258</v>
+        <v>94</v>
       </c>
       <c r="E55" s="6"/>
       <c r="F55" s="6"/>
@@ -3029,14 +3007,16 @@
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
-        <v>286</v>
-      </c>
-      <c r="B56" s="4"/>
+        <v>309</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="C56" s="4">
-        <v>400007</v>
+        <v>200008</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>259</v>
+        <v>93</v>
       </c>
       <c r="E56" s="6"/>
       <c r="F56" s="6"/>
@@ -3054,16 +3034,16 @@
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>317</v>
+        <v>14</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="C57" s="4">
-        <v>400009</v>
+        <v>500003</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="E57" s="6"/>
       <c r="F57" s="6"/>
@@ -3081,16 +3061,16 @@
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>317</v>
+        <v>14</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>318</v>
+        <v>17</v>
       </c>
       <c r="C58" s="4">
-        <v>400011</v>
+        <v>500004</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>300</v>
+        <v>104</v>
       </c>
       <c r="E58" s="6"/>
       <c r="F58" s="6"/>
@@ -3108,14 +3088,16 @@
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
-        <v>286</v>
-      </c>
-      <c r="B59" s="4"/>
+        <v>14</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>312</v>
+      </c>
       <c r="C59" s="4">
-        <v>400012</v>
+        <v>500009</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>118</v>
+        <v>295</v>
       </c>
       <c r="E59" s="6"/>
       <c r="F59" s="6"/>
@@ -3133,16 +3115,16 @@
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>31</v>
+        <v>285</v>
       </c>
       <c r="C60" s="4">
-        <v>400013</v>
+        <v>500010</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>120</v>
+        <v>296</v>
       </c>
       <c r="E60" s="6"/>
       <c r="F60" s="6"/>
@@ -3160,16 +3142,16 @@
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>31</v>
+        <v>285</v>
       </c>
       <c r="C61" s="4">
-        <v>400014</v>
+        <v>500011</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>119</v>
+        <v>297</v>
       </c>
       <c r="E61" s="6"/>
       <c r="F61" s="6"/>
@@ -3190,13 +3172,13 @@
         <v>14</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>319</v>
+        <v>17</v>
       </c>
       <c r="C62" s="4">
-        <v>500003</v>
+        <v>500012</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>301</v>
+        <v>103</v>
       </c>
       <c r="E62" s="6"/>
       <c r="F62" s="6"/>
@@ -3217,13 +3199,13 @@
         <v>14</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>17</v>
+        <v>285</v>
       </c>
       <c r="C63" s="4">
-        <v>500004</v>
+        <v>500013</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>104</v>
+        <v>298</v>
       </c>
       <c r="E63" s="6"/>
       <c r="F63" s="6"/>
@@ -3244,13 +3226,13 @@
         <v>14</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>319</v>
+        <v>18</v>
       </c>
       <c r="C64" s="4">
-        <v>500009</v>
+        <v>500014</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>302</v>
+        <v>105</v>
       </c>
       <c r="E64" s="6"/>
       <c r="F64" s="6"/>
@@ -3268,16 +3250,16 @@
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
-        <v>287</v>
+        <v>14</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C65" s="4">
-        <v>500010</v>
+        <v>500018</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="E65" s="6"/>
       <c r="F65" s="6"/>
@@ -3295,16 +3277,16 @@
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
-        <v>287</v>
+        <v>14</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>288</v>
+        <v>16</v>
       </c>
       <c r="C66" s="4">
-        <v>500011</v>
+        <v>500019</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>304</v>
+        <v>102</v>
       </c>
       <c r="E66" s="6"/>
       <c r="F66" s="6"/>
@@ -3325,13 +3307,13 @@
         <v>14</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C67" s="4">
-        <v>500012</v>
+        <v>500020</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E67" s="6"/>
       <c r="F67" s="6"/>
@@ -3349,16 +3331,16 @@
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
-        <v>287</v>
+        <v>14</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>288</v>
+        <v>16</v>
       </c>
       <c r="C68" s="4">
-        <v>500013</v>
+        <v>500021</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>305</v>
+        <v>101</v>
       </c>
       <c r="E68" s="6"/>
       <c r="F68" s="6"/>
@@ -3379,13 +3361,13 @@
         <v>14</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C69" s="4">
-        <v>500014</v>
+        <v>500025</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
@@ -3403,16 +3385,16 @@
     </row>
     <row r="70" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
-        <v>287</v>
+        <v>14</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C70" s="4">
-        <v>500018</v>
+        <v>500026</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="E70" s="6"/>
       <c r="F70" s="6"/>
@@ -3433,13 +3415,13 @@
         <v>14</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C71" s="4">
-        <v>500019</v>
+        <v>500027</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>102</v>
+        <v>165</v>
       </c>
       <c r="E71" s="6"/>
       <c r="F71" s="6"/>
@@ -3457,19 +3439,21 @@
     </row>
     <row r="72" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C72" s="4">
-        <v>500020</v>
+        <v>600001</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="E72" s="6"/>
-      <c r="F72" s="6"/>
+      <c r="F72" s="6" t="s">
+        <v>284</v>
+      </c>
       <c r="G72" s="6"/>
       <c r="H72" s="6"/>
       <c r="I72" s="6"/>
@@ -3484,24 +3468,32 @@
     </row>
     <row r="73" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C73" s="4">
-        <v>500021</v>
+        <v>600002</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="E73" s="6"/>
-      <c r="F73" s="6"/>
-      <c r="G73" s="6"/>
+      <c r="F73" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="G73" s="6" t="s">
+        <v>281</v>
+      </c>
       <c r="H73" s="6"/>
       <c r="I73" s="6"/>
-      <c r="J73" s="6"/>
-      <c r="K73" s="6"/>
+      <c r="J73" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="K73" s="6" t="s">
+        <v>283</v>
+      </c>
       <c r="L73" s="6"/>
       <c r="M73" s="6"/>
       <c r="N73" s="6"/>
@@ -3511,16 +3503,16 @@
     </row>
     <row r="74" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C74" s="4">
-        <v>500025</v>
+        <v>600003</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="6"/>
@@ -3538,16 +3530,16 @@
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
-        <v>287</v>
+        <v>19</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>288</v>
+        <v>21</v>
       </c>
       <c r="C75" s="4">
-        <v>500026</v>
+        <v>600004</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>307</v>
+        <v>108</v>
       </c>
       <c r="E75" s="6"/>
       <c r="F75" s="6"/>
@@ -3565,20 +3557,24 @@
     </row>
     <row r="76" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C76" s="4">
-        <v>500027</v>
+        <v>600005</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>165</v>
+        <v>112</v>
       </c>
       <c r="E76" s="6"/>
-      <c r="F76" s="6"/>
-      <c r="G76" s="6"/>
+      <c r="F76" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="G76" s="6" t="s">
+        <v>266</v>
+      </c>
       <c r="H76" s="6"/>
       <c r="I76" s="6"/>
       <c r="J76" s="6"/>
@@ -3595,18 +3591,18 @@
         <v>19</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C77" s="4">
-        <v>600001</v>
+        <v>600006</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="E77" s="6"/>
-      <c r="F77" s="6" t="s">
-        <v>284</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="F77" s="6"/>
       <c r="G77" s="6"/>
       <c r="H77" s="6"/>
       <c r="I77" s="6"/>
@@ -3624,29 +3620,21 @@
         <v>19</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C78" s="4">
-        <v>600002</v>
+        <v>600007</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E78" s="6"/>
-      <c r="F78" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="G78" s="6" t="s">
-        <v>281</v>
-      </c>
+      <c r="F78" s="6"/>
+      <c r="G78" s="6"/>
       <c r="H78" s="6"/>
       <c r="I78" s="6"/>
-      <c r="J78" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="K78" s="6" t="s">
-        <v>283</v>
-      </c>
+      <c r="J78" s="6"/>
+      <c r="K78" s="6"/>
       <c r="L78" s="6"/>
       <c r="M78" s="6"/>
       <c r="N78" s="6"/>
@@ -3659,21 +3647,29 @@
         <v>19</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C79" s="4">
-        <v>600003</v>
+        <v>600008</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E79" s="6"/>
-      <c r="F79" s="6"/>
-      <c r="G79" s="6"/>
+      <c r="F79" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="G79" s="6" t="s">
+        <v>281</v>
+      </c>
       <c r="H79" s="6"/>
       <c r="I79" s="6"/>
-      <c r="J79" s="6"/>
-      <c r="K79" s="6"/>
+      <c r="J79" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="K79" s="6" t="s">
+        <v>283</v>
+      </c>
       <c r="L79" s="6"/>
       <c r="M79" s="6"/>
       <c r="N79" s="6"/>
@@ -3686,21 +3682,29 @@
         <v>19</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C80" s="4">
-        <v>600004</v>
+        <v>600009</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="E80" s="6"/>
-      <c r="F80" s="6"/>
-      <c r="G80" s="6"/>
+      <c r="F80" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="G80" s="6" t="s">
+        <v>281</v>
+      </c>
       <c r="H80" s="6"/>
       <c r="I80" s="6"/>
-      <c r="J80" s="6"/>
-      <c r="K80" s="6"/>
+      <c r="J80" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="K80" s="6" t="s">
+        <v>283</v>
+      </c>
       <c r="L80" s="6"/>
       <c r="M80" s="6"/>
       <c r="N80" s="6"/>
@@ -3712,22 +3716,16 @@
       <c r="A81" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B81" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="B81" s="4"/>
       <c r="C81" s="4">
-        <v>600005</v>
+        <v>600010</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="E81" s="6"/>
-      <c r="F81" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="G81" s="6" t="s">
-        <v>266</v>
-      </c>
+      <c r="F81" s="6"/>
+      <c r="G81" s="6"/>
       <c r="H81" s="6"/>
       <c r="I81" s="6"/>
       <c r="J81" s="6"/>
@@ -3744,23 +3742,29 @@
         <v>19</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C82" s="4">
-        <v>600006</v>
+        <v>600011</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="E82" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="F82" s="6"/>
-      <c r="G82" s="6"/>
+        <v>107</v>
+      </c>
+      <c r="E82" s="6"/>
+      <c r="F82" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>281</v>
+      </c>
       <c r="H82" s="6"/>
       <c r="I82" s="6"/>
-      <c r="J82" s="6"/>
-      <c r="K82" s="6"/>
+      <c r="J82" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>283</v>
+      </c>
       <c r="L82" s="6"/>
       <c r="M82" s="6"/>
       <c r="N82" s="6"/>
@@ -3772,14 +3776,12 @@
       <c r="A83" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B83" s="4" t="s">
-        <v>23</v>
-      </c>
+      <c r="B83" s="4"/>
       <c r="C83" s="4">
-        <v>600007</v>
+        <v>600012</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>110</v>
+        <v>157</v>
       </c>
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
@@ -3797,32 +3799,24 @@
     </row>
     <row r="84" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="C84" s="4">
-        <v>600008</v>
+        <v>400000</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="E84" s="6"/>
-      <c r="F84" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="G84" s="6" t="s">
-        <v>281</v>
-      </c>
+      <c r="F84" s="6"/>
+      <c r="G84" s="6"/>
       <c r="H84" s="6"/>
       <c r="I84" s="6"/>
-      <c r="J84" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="K84" s="6" t="s">
-        <v>283</v>
-      </c>
+      <c r="J84" s="6"/>
+      <c r="K84" s="6"/>
       <c r="L84" s="6"/>
       <c r="M84" s="6"/>
       <c r="N84" s="6"/>
@@ -3832,32 +3826,24 @@
     </row>
     <row r="85" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C85" s="4">
-        <v>600009</v>
+        <v>400001</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E85" s="6"/>
-      <c r="F85" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="G85" s="6" t="s">
-        <v>281</v>
-      </c>
+      <c r="F85" s="6"/>
+      <c r="G85" s="6"/>
       <c r="H85" s="6"/>
       <c r="I85" s="6"/>
-      <c r="J85" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="K85" s="6" t="s">
-        <v>283</v>
-      </c>
+      <c r="J85" s="6"/>
+      <c r="K85" s="6"/>
       <c r="L85" s="6"/>
       <c r="M85" s="6"/>
       <c r="N85" s="6"/>
@@ -3867,14 +3853,16 @@
     </row>
     <row r="86" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
-        <v>289</v>
-      </c>
-      <c r="B86" s="4"/>
+        <v>29</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>32</v>
+      </c>
       <c r="C86" s="4">
-        <v>600010</v>
+        <v>400002</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="E86" s="6"/>
       <c r="F86" s="6"/>
@@ -3892,32 +3880,24 @@
     </row>
     <row r="87" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C87" s="4">
-        <v>600011</v>
+        <v>400003</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E87" s="6"/>
-      <c r="F87" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="G87" s="6" t="s">
-        <v>281</v>
-      </c>
+      <c r="F87" s="6"/>
+      <c r="G87" s="6"/>
       <c r="H87" s="6"/>
       <c r="I87" s="6"/>
-      <c r="J87" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="K87" s="6" t="s">
-        <v>283</v>
-      </c>
+      <c r="J87" s="6"/>
+      <c r="K87" s="6"/>
       <c r="L87" s="6"/>
       <c r="M87" s="6"/>
       <c r="N87" s="6"/>
@@ -3927,14 +3907,14 @@
     </row>
     <row r="88" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
-        <v>289</v>
+        <v>29</v>
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="4">
-        <v>600012</v>
+        <v>400004</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>157</v>
+        <v>258</v>
       </c>
       <c r="E88" s="6"/>
       <c r="F88" s="6"/>
@@ -3952,16 +3932,14 @@
     </row>
     <row r="89" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B89" s="4" t="s">
-        <v>38</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="B89" s="4"/>
       <c r="C89" s="4">
-        <v>700001</v>
+        <v>400007</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>135</v>
+        <v>259</v>
       </c>
       <c r="E89" s="6"/>
       <c r="F89" s="6"/>
@@ -3979,16 +3957,14 @@
     </row>
     <row r="90" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B90" s="4" t="s">
-        <v>38</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="B90" s="4"/>
       <c r="C90" s="4">
-        <v>700002</v>
+        <v>400012</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="E90" s="6"/>
       <c r="F90" s="6"/>
@@ -4006,16 +3982,16 @@
     </row>
     <row r="91" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C91" s="4">
-        <v>700003</v>
+        <v>400013</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="E91" s="6"/>
       <c r="F91" s="6"/>
@@ -4033,16 +4009,16 @@
     </row>
     <row r="92" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C92" s="4">
-        <v>700004</v>
+        <v>400014</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="E92" s="6"/>
       <c r="F92" s="6"/>
@@ -4060,16 +4036,16 @@
     </row>
     <row r="93" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>37</v>
+        <v>308</v>
       </c>
       <c r="C93" s="4">
-        <v>700005</v>
+        <v>300001</v>
       </c>
       <c r="D93" s="5" t="s">
-        <v>129</v>
+        <v>290</v>
       </c>
       <c r="E93" s="6"/>
       <c r="F93" s="6"/>
@@ -4087,16 +4063,16 @@
     </row>
     <row r="94" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C94" s="4">
-        <v>700006</v>
+        <v>300002</v>
       </c>
       <c r="D94" s="5" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="E94" s="6"/>
       <c r="F94" s="6"/>
@@ -4114,16 +4090,16 @@
     </row>
     <row r="95" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A95" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C95" s="4">
-        <v>700007</v>
+        <v>300003</v>
       </c>
       <c r="D95" s="5" t="s">
-        <v>128</v>
+        <v>291</v>
       </c>
       <c r="E95" s="6"/>
       <c r="F95" s="6"/>
@@ -4144,13 +4120,13 @@
         <v>35</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C96" s="4">
-        <v>700008</v>
+        <v>700001</v>
       </c>
       <c r="D96" s="5" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E96" s="6"/>
       <c r="F96" s="6"/>
@@ -4168,16 +4144,16 @@
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
-        <v>290</v>
+        <v>35</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>292</v>
+        <v>38</v>
       </c>
       <c r="C97" s="4">
-        <v>700009</v>
+        <v>700002</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>308</v>
+        <v>132</v>
       </c>
       <c r="E97" s="6"/>
       <c r="F97" s="6"/>
@@ -4195,16 +4171,16 @@
     </row>
     <row r="98" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
-        <v>290</v>
+        <v>35</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>291</v>
+        <v>38</v>
       </c>
       <c r="C98" s="4">
-        <v>700010</v>
+        <v>700003</v>
       </c>
       <c r="D98" s="5" t="s">
-        <v>309</v>
+        <v>134</v>
       </c>
       <c r="E98" s="6"/>
       <c r="F98" s="6"/>
@@ -4222,16 +4198,16 @@
     </row>
     <row r="99" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A99" s="4" t="s">
-        <v>290</v>
+        <v>35</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>291</v>
+        <v>38</v>
       </c>
       <c r="C99" s="4">
-        <v>700011</v>
+        <v>700004</v>
       </c>
       <c r="D99" s="5" t="s">
-        <v>310</v>
+        <v>133</v>
       </c>
       <c r="E99" s="6"/>
       <c r="F99" s="6"/>
@@ -4249,16 +4225,16 @@
     </row>
     <row r="100" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A100" s="4" t="s">
-        <v>290</v>
+        <v>35</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>291</v>
+        <v>37</v>
       </c>
       <c r="C100" s="4">
-        <v>700012</v>
+        <v>700005</v>
       </c>
       <c r="D100" s="5" t="s">
-        <v>311</v>
+        <v>129</v>
       </c>
       <c r="E100" s="6"/>
       <c r="F100" s="6"/>
@@ -4279,13 +4255,13 @@
         <v>35</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C101" s="4">
-        <v>700013</v>
+        <v>700006</v>
       </c>
       <c r="D101" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E101" s="6"/>
       <c r="F101" s="6"/>
@@ -4306,13 +4282,13 @@
         <v>35</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C102" s="4">
-        <v>700014</v>
+        <v>700007</v>
       </c>
       <c r="D102" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E102" s="6"/>
       <c r="F102" s="6"/>
@@ -4333,13 +4309,13 @@
         <v>35</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C103" s="4">
-        <v>700015</v>
+        <v>700008</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E103" s="6"/>
       <c r="F103" s="6"/>
@@ -4360,13 +4336,13 @@
         <v>35</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>36</v>
+        <v>287</v>
       </c>
       <c r="C104" s="4">
-        <v>700016</v>
+        <v>700009</v>
       </c>
       <c r="D104" s="5" t="s">
-        <v>127</v>
+        <v>301</v>
       </c>
       <c r="E104" s="6"/>
       <c r="F104" s="6"/>
@@ -4387,13 +4363,13 @@
         <v>35</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>39</v>
+        <v>286</v>
       </c>
       <c r="C105" s="4">
-        <v>700017</v>
+        <v>700010</v>
       </c>
       <c r="D105" s="5" t="s">
-        <v>138</v>
+        <v>302</v>
       </c>
       <c r="E105" s="6"/>
       <c r="F105" s="6"/>
@@ -4414,13 +4390,13 @@
         <v>35</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>39</v>
+        <v>286</v>
       </c>
       <c r="C106" s="4">
-        <v>700018</v>
+        <v>700011</v>
       </c>
       <c r="D106" s="5" t="s">
-        <v>137</v>
+        <v>303</v>
       </c>
       <c r="E106" s="6"/>
       <c r="F106" s="6"/>
@@ -4441,13 +4417,13 @@
         <v>35</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>39</v>
+        <v>286</v>
       </c>
       <c r="C107" s="4">
-        <v>700019</v>
+        <v>700012</v>
       </c>
       <c r="D107" s="5" t="s">
-        <v>136</v>
+        <v>304</v>
       </c>
       <c r="E107" s="6"/>
       <c r="F107" s="6"/>
@@ -4468,13 +4444,13 @@
         <v>35</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C108" s="4">
-        <v>700020</v>
+        <v>700013</v>
       </c>
       <c r="D108" s="5" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="E108" s="6"/>
       <c r="F108" s="6"/>
@@ -4495,13 +4471,13 @@
         <v>35</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C109" s="4">
-        <v>700021</v>
+        <v>700014</v>
       </c>
       <c r="D109" s="5" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="E109" s="6"/>
       <c r="F109" s="6"/>
@@ -4522,13 +4498,13 @@
         <v>35</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C110" s="4">
-        <v>700022</v>
+        <v>700015</v>
       </c>
       <c r="D110" s="5" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="E110" s="6"/>
       <c r="F110" s="6"/>
@@ -4549,13 +4525,13 @@
         <v>35</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C111" s="4">
-        <v>700023</v>
+        <v>700016</v>
       </c>
       <c r="D111" s="5" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="E111" s="6"/>
       <c r="F111" s="6"/>
@@ -4579,10 +4555,10 @@
         <v>39</v>
       </c>
       <c r="C112" s="4">
-        <v>700024</v>
+        <v>700017</v>
       </c>
       <c r="D112" s="5" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E112" s="6"/>
       <c r="F112" s="6"/>
@@ -4600,34 +4576,24 @@
     </row>
     <row r="113" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C113" s="4">
-        <v>900000</v>
+        <v>700018</v>
       </c>
       <c r="D113" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="E113" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="F113" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="G113" s="6" t="s">
-        <v>269</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="E113" s="6"/>
+      <c r="F113" s="6"/>
+      <c r="G113" s="6"/>
       <c r="H113" s="6"/>
       <c r="I113" s="6"/>
-      <c r="J113" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="K113" s="6" t="s">
-        <v>275</v>
-      </c>
+      <c r="J113" s="6"/>
+      <c r="K113" s="6"/>
       <c r="L113" s="6"/>
       <c r="M113" s="6"/>
       <c r="N113" s="6"/>
@@ -4637,34 +4603,24 @@
     </row>
     <row r="114" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A114" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C114" s="4">
-        <v>900001</v>
+        <v>700019</v>
       </c>
       <c r="D114" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="E114" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="F114" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="G114" s="6" t="s">
-        <v>269</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="E114" s="6"/>
+      <c r="F114" s="6"/>
+      <c r="G114" s="6"/>
       <c r="H114" s="6"/>
       <c r="I114" s="6"/>
-      <c r="J114" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="K114" s="6" t="s">
-        <v>275</v>
-      </c>
+      <c r="J114" s="6"/>
+      <c r="K114" s="6"/>
       <c r="L114" s="6"/>
       <c r="M114" s="6"/>
       <c r="N114" s="6"/>
@@ -4674,16 +4630,16 @@
     </row>
     <row r="115" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A115" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C115" s="4">
-        <v>900002</v>
+        <v>700020</v>
       </c>
       <c r="D115" s="5" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="E115" s="6"/>
       <c r="F115" s="6"/>
@@ -4701,34 +4657,24 @@
     </row>
     <row r="116" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A116" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C116" s="4">
-        <v>900003</v>
+        <v>700021</v>
       </c>
       <c r="D116" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="E116" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="F116" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="G116" s="6" t="s">
-        <v>269</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="E116" s="6"/>
+      <c r="F116" s="6"/>
+      <c r="G116" s="6"/>
       <c r="H116" s="6"/>
       <c r="I116" s="6"/>
-      <c r="J116" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="K116" s="6" t="s">
-        <v>275</v>
-      </c>
+      <c r="J116" s="6"/>
+      <c r="K116" s="6"/>
       <c r="L116" s="6"/>
       <c r="M116" s="6"/>
       <c r="N116" s="6"/>
@@ -4738,16 +4684,16 @@
     </row>
     <row r="117" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A117" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C117" s="4">
-        <v>900004</v>
+        <v>700022</v>
       </c>
       <c r="D117" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E117" s="6"/>
       <c r="F117" s="6"/>
@@ -4765,16 +4711,16 @@
     </row>
     <row r="118" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A118" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C118" s="4">
-        <v>900005</v>
+        <v>700023</v>
       </c>
       <c r="D118" s="5" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="E118" s="6"/>
       <c r="F118" s="6"/>
@@ -4792,16 +4738,16 @@
     </row>
     <row r="119" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A119" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C119" s="4">
-        <v>900006</v>
+        <v>700024</v>
       </c>
       <c r="D119" s="5" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E119" s="6"/>
       <c r="F119" s="6"/>
@@ -4822,21 +4768,31 @@
         <v>40</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C120" s="4">
-        <v>900007</v>
+        <v>900000</v>
       </c>
       <c r="D120" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="E120" s="6"/>
-      <c r="F120" s="6"/>
-      <c r="G120" s="6"/>
+        <v>152</v>
+      </c>
+      <c r="E120" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="F120" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="G120" s="6" t="s">
+        <v>269</v>
+      </c>
       <c r="H120" s="6"/>
       <c r="I120" s="6"/>
-      <c r="J120" s="6"/>
-      <c r="K120" s="6"/>
+      <c r="J120" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="K120" s="6" t="s">
+        <v>275</v>
+      </c>
       <c r="L120" s="6"/>
       <c r="M120" s="6"/>
       <c r="N120" s="6"/>
@@ -4849,21 +4805,31 @@
         <v>40</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C121" s="4">
-        <v>900008</v>
+        <v>900001</v>
       </c>
       <c r="D121" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="E121" s="6"/>
-      <c r="F121" s="6"/>
-      <c r="G121" s="6"/>
+        <v>153</v>
+      </c>
+      <c r="E121" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="F121" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="G121" s="6" t="s">
+        <v>269</v>
+      </c>
       <c r="H121" s="6"/>
       <c r="I121" s="6"/>
-      <c r="J121" s="6"/>
-      <c r="K121" s="6"/>
+      <c r="J121" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="K121" s="6" t="s">
+        <v>275</v>
+      </c>
       <c r="L121" s="6"/>
       <c r="M121" s="6"/>
       <c r="N121" s="6"/>
@@ -4876,13 +4842,13 @@
         <v>40</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C122" s="4">
-        <v>900009</v>
+        <v>900002</v>
       </c>
       <c r="D122" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E122" s="6"/>
       <c r="F122" s="6"/>
@@ -4900,24 +4866,34 @@
     </row>
     <row r="123" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A123" s="4" t="s">
-        <v>293</v>
+        <v>40</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>294</v>
+        <v>46</v>
       </c>
       <c r="C123" s="4">
-        <v>900010</v>
+        <v>900003</v>
       </c>
       <c r="D123" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="E123" s="6"/>
-      <c r="F123" s="6"/>
-      <c r="G123" s="6"/>
+        <v>151</v>
+      </c>
+      <c r="E123" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="F123" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="G123" s="6" t="s">
+        <v>269</v>
+      </c>
       <c r="H123" s="6"/>
       <c r="I123" s="6"/>
-      <c r="J123" s="6"/>
-      <c r="K123" s="6"/>
+      <c r="J123" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="K123" s="6" t="s">
+        <v>275</v>
+      </c>
       <c r="L123" s="6"/>
       <c r="M123" s="6"/>
       <c r="N123" s="6"/>
@@ -4927,16 +4903,16 @@
     </row>
     <row r="124" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A124" s="4" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C124" s="4" t="s">
-        <v>62</v>
+        <v>41</v>
+      </c>
+      <c r="C124" s="4">
+        <v>900004</v>
       </c>
       <c r="D124" s="5" t="s">
-        <v>63</v>
+        <v>144</v>
       </c>
       <c r="E124" s="6"/>
       <c r="F124" s="6"/>
@@ -4954,16 +4930,16 @@
     </row>
     <row r="125" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C125" s="4" t="s">
-        <v>82</v>
+        <v>41</v>
+      </c>
+      <c r="C125" s="4">
+        <v>900005</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="E125" s="6"/>
       <c r="F125" s="6"/>
@@ -4981,16 +4957,16 @@
     </row>
     <row r="126" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A126" s="4" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C126" s="4" t="s">
-        <v>78</v>
+        <v>42</v>
+      </c>
+      <c r="C126" s="4">
+        <v>900006</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="E126" s="6"/>
       <c r="F126" s="6"/>
@@ -5008,16 +4984,16 @@
     </row>
     <row r="127" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A127" s="4" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C127" s="4" t="s">
-        <v>84</v>
+        <v>41</v>
+      </c>
+      <c r="C127" s="4">
+        <v>900007</v>
       </c>
       <c r="D127" s="5" t="s">
-        <v>85</v>
+        <v>146</v>
       </c>
       <c r="E127" s="6"/>
       <c r="F127" s="6"/>
@@ -5035,16 +5011,16 @@
     </row>
     <row r="128" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C128" s="4" t="s">
-        <v>80</v>
+        <v>43</v>
+      </c>
+      <c r="C128" s="4">
+        <v>900008</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>81</v>
+        <v>148</v>
       </c>
       <c r="E128" s="6"/>
       <c r="F128" s="6"/>
@@ -5062,16 +5038,16 @@
     </row>
     <row r="129" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A129" s="4" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C129" s="4" t="s">
-        <v>86</v>
+        <v>45</v>
+      </c>
+      <c r="C129" s="4">
+        <v>900009</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>87</v>
+        <v>150</v>
       </c>
       <c r="E129" s="6"/>
       <c r="F129" s="6"/>
@@ -5089,16 +5065,16 @@
     </row>
     <row r="130" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A130" s="4" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C130" s="4" t="s">
-        <v>88</v>
+        <v>43</v>
+      </c>
+      <c r="C130" s="4">
+        <v>900010</v>
       </c>
       <c r="D130" s="5" t="s">
-        <v>89</v>
+        <v>305</v>
       </c>
       <c r="E130" s="6"/>
       <c r="F130" s="6"/>
@@ -5114,8 +5090,39 @@
       <c r="P130" s="6"/>
       <c r="Q130" s="6"/>
     </row>
+    <row r="131" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A131" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="C131" s="4">
+        <v>900011</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="E131" s="6"/>
+      <c r="F131" s="6"/>
+      <c r="G131" s="6"/>
+      <c r="H131" s="6"/>
+      <c r="I131" s="6"/>
+      <c r="J131" s="6"/>
+      <c r="K131" s="6"/>
+      <c r="L131" s="6"/>
+      <c r="M131" s="6"/>
+      <c r="N131" s="6"/>
+      <c r="O131" s="6"/>
+      <c r="P131" s="6"/>
+      <c r="Q131" s="6"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:Q130" xr:uid="{9157580D-EE50-43E2-A76D-B56C98A189DD}"/>
+  <autoFilter ref="A2:Q131" xr:uid="{9157580D-EE50-43E2-A76D-B56C98A189DD}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:Q131">
+      <sortCondition ref="A2:A131"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>